<commit_message>
docs/feat: update Excel with V8 results (Correctness: 50.0%, Relevancy: 98.0%) and apply V9 config (Epochs 1, Rank 16)
</commit_message>
<xml_diff>
--- a/finetune-results.xlsx
+++ b/finetune-results.xlsx
@@ -1410,6 +1410,7 @@
     <col width="25" customWidth="1" style="18" min="8" max="8"/>
     <col width="25" customWidth="1" style="18" min="9" max="9"/>
     <col width="25" customWidth="1" style="18" min="10" max="10"/>
+    <col width="25" customWidth="1" style="18" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1506,7 +1507,11 @@
           <t>VERSION 8 (V7 + Epochs=2)</t>
         </is>
       </c>
-      <c r="K6" s="28" t="n"/>
+      <c r="K6" s="27" t="inlineStr">
+        <is>
+          <t>VERSION 9 (V7 + Rank=16)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
@@ -1556,10 +1561,14 @@
       </c>
       <c r="J7" s="31" t="inlineStr">
         <is>
+          <t>98.0%</t>
+        </is>
+      </c>
+      <c r="K7" s="31" t="inlineStr">
+        <is>
           <t>[PENDING]</t>
         </is>
       </c>
-      <c r="K7" s="28" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
@@ -1607,12 +1616,16 @@
           <t>50.0%</t>
         </is>
       </c>
-      <c r="J8" s="31" t="inlineStr">
+      <c r="J8" s="33" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+      <c r="K8" s="31" t="inlineStr">
         <is>
           <t>[PENDING]</t>
         </is>
       </c>
-      <c r="K8" s="28" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
@@ -1665,7 +1678,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="K9" s="28" t="n"/>
+      <c r="K9" s="25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="29" t="inlineStr">
@@ -1718,7 +1735,11 @@
           <t>1e-5 (0.00001)</t>
         </is>
       </c>
-      <c r="K10" s="28" t="n"/>
+      <c r="K10" s="25" t="inlineStr">
+        <is>
+          <t>1e-5 (0.00001)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
@@ -1771,7 +1792,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="K11" s="28" t="n"/>
+      <c r="K11" s="25" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
@@ -1824,7 +1849,11 @@
           <t>1024</t>
         </is>
       </c>
-      <c r="K12" s="28" t="n"/>
+      <c r="K12" s="25" t="inlineStr">
+        <is>
+          <t>1024</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
@@ -1874,14 +1903,18 @@
       </c>
       <c r="J13" s="30" t="inlineStr">
         <is>
-          <t>Single variable test (Epochs=2)</t>
-        </is>
-      </c>
-      <c r="K13" s="28" t="n"/>
+          <t>Marginal/Flat: Epochs=2 did not improve correctness</t>
+        </is>
+      </c>
+      <c r="K13" s="25" t="inlineStr">
+        <is>
+          <t>Single variable test (r=16)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs/feat: update Excel with V9 results (Correctness: 35.2%, Relevancy: 98.1%) and apply V10 config (Epochs 1, LR 5e-6)
</commit_message>
<xml_diff>
--- a/finetune-results.xlsx
+++ b/finetune-results.xlsx
@@ -1397,7 +1397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.6"/>
   <cols>
     <col width="30" customWidth="1" style="18" min="1" max="1"/>
@@ -1411,6 +1411,7 @@
     <col width="25" customWidth="1" style="18" min="9" max="9"/>
     <col width="25" customWidth="1" style="18" min="10" max="10"/>
     <col width="25" customWidth="1" style="18" min="11" max="11"/>
+    <col width="25" customWidth="1" style="18" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1512,6 +1513,11 @@
           <t>VERSION 9 (V7 + Rank=16)</t>
         </is>
       </c>
+      <c r="L6" s="27" t="inlineStr">
+        <is>
+          <t>VERSION 10 (V7 + Slower LR)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
@@ -1566,6 +1572,11 @@
       </c>
       <c r="K7" s="31" t="inlineStr">
         <is>
+          <t>98.1%</t>
+        </is>
+      </c>
+      <c r="L7" s="31" t="inlineStr">
+        <is>
           <t>[PENDING]</t>
         </is>
       </c>
@@ -1621,7 +1632,12 @@
           <t>50.0%</t>
         </is>
       </c>
-      <c r="K8" s="31" t="inlineStr">
+      <c r="K8" s="33" t="inlineStr">
+        <is>
+          <t>35.2%</t>
+        </is>
+      </c>
+      <c r="L8" s="31" t="inlineStr">
         <is>
           <t>[PENDING]</t>
         </is>
@@ -1683,6 +1699,11 @@
           <t>1</t>
         </is>
       </c>
+      <c r="L9" s="25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="29" t="inlineStr">
@@ -1740,6 +1761,11 @@
           <t>1e-5 (0.00001)</t>
         </is>
       </c>
+      <c r="L10" s="25" t="inlineStr">
+        <is>
+          <t>5e-6 (0.000005)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
@@ -1797,6 +1823,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="L11" s="25" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
@@ -1854,6 +1885,11 @@
           <t>1024</t>
         </is>
       </c>
+      <c r="L12" s="25" t="inlineStr">
+        <is>
+          <t>1024</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
@@ -1908,13 +1944,18 @@
       </c>
       <c r="K13" s="25" t="inlineStr">
         <is>
-          <t>Single variable test (r=16)</t>
+          <t>Failed: Higher rank caused overfitting</t>
+        </is>
+      </c>
+      <c r="L13" s="25" t="inlineStr">
+        <is>
+          <t>Single variable test (LR=5e-6)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:L1"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>